<commit_message>
Bundled better assembler and fixed errors in the CPU
</commit_message>
<xml_diff>
--- a/Assembly/Spec Sheets/CPU Instruction set.xlsx
+++ b/Assembly/Spec Sheets/CPU Instruction set.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="109">
   <si>
     <t xml:space="preserve">HEX</t>
   </si>
@@ -32,12 +32,21 @@
     <t xml:space="preserve">DESCRIPTION</t>
   </si>
   <si>
+    <t xml:space="preserve">ALIAS(ES)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">48 bit per inst.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ADC</t>
   </si>
   <si>
     <t xml:space="preserve">Adds &lt;tar&gt; to &lt;sel&gt;, outputs to &lt;slc&gt;; carry is outputted to CR</t>
   </si>
   <si>
+    <t xml:space="preserve">8 bit loaded at a time</t>
+  </si>
+  <si>
     <t xml:space="preserve">ADD</t>
   </si>
   <si>
@@ -71,7 +80,10 @@
     <t xml:space="preserve">UNA</t>
   </si>
   <si>
-    <t xml:space="preserve">Unallocated / No Operation (NOP alias)</t>
+    <t xml:space="preserve">Unallocated / No Operation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOP</t>
   </si>
   <si>
     <t xml:space="preserve">PUS</t>
@@ -152,12 +164,18 @@
     <t xml:space="preserve">Sets &lt;slc&gt; to &lt;sel&gt; </t>
   </si>
   <si>
+    <t xml:space="preserve">SET, WRT, LDR</t>
+  </si>
+  <si>
     <t xml:space="preserve">JSR</t>
   </si>
   <si>
     <t xml:space="preserve">Jumps to a subroutine; Pushes to stack</t>
   </si>
   <si>
+    <t xml:space="preserve">JMP</t>
+  </si>
+  <si>
     <t xml:space="preserve">RET</t>
   </si>
   <si>
@@ -170,34 +188,124 @@
     <t xml:space="preserve">Halt until the next interrupt</t>
   </si>
   <si>
+    <t xml:space="preserve">STP</t>
+  </si>
+  <si>
     <t xml:space="preserve">CMP</t>
   </si>
   <si>
     <t xml:space="preserve">SBB but only CR output</t>
   </si>
   <si>
+    <t xml:space="preserve">DIF</t>
+  </si>
+  <si>
     <t xml:space="preserve">SHL</t>
   </si>
   <si>
-    <t xml:space="preserve">Shifts &lt;tar&gt; left; uses &lt;slc&gt;</t>
+    <t xml:space="preserve">Shifts &lt;tar&gt; left &lt;sel&gt; times; uses &lt;slc&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">ROL</t>
   </si>
   <si>
-    <t xml:space="preserve">Rotates &lt;tar&gt; left; uses &lt;slc&gt;</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Rotates &lt;tar&gt; left </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> &lt;sel&gt; times</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">; uses &lt;slc&gt;</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">SHR</t>
   </si>
   <si>
-    <t xml:space="preserve">shifts &lt;tar&gt; right; uses &lt;slc&gt;</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">shifts &lt;tar&gt; right </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> &lt;sel&gt; times</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">; uses &lt;slc&gt;</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">ROR</t>
   </si>
   <si>
-    <t xml:space="preserve">Rotates &lt;tar&gt; right; uses &lt;slc&gt;</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Rotates &lt;tar&gt; right </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> &lt;sel&gt; times</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">; uses &lt;slc&gt;</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">i. HEX</t>
@@ -346,7 +454,19 @@
     <t xml:space="preserve">Immediate Value</t>
   </si>
   <si>
+    <t xml:space="preserve">Read, N/A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VOID</t>
+  </si>
+  <si>
     <t xml:space="preserve">N/A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -360,7 +480,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -396,6 +516,12 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="11"/>
@@ -453,7 +579,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -466,6 +592,10 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -474,16 +604,16 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -613,37 +743,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4285f4"/>
+        <a:srgbClr val="4285F4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ea4335"/>
+        <a:srgbClr val="EA4335"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="fbbc04"/>
+        <a:srgbClr val="FBBC04"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="34a853"/>
+        <a:srgbClr val="34A853"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="ff6d01"/>
+        <a:srgbClr val="FF6D01"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="46bdc6"/>
+        <a:srgbClr val="46BDC6"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="1155cc"/>
+        <a:srgbClr val="1155CC"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="1155cc"/>
+        <a:srgbClr val="1155CC"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -716,12 +846,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="70.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="8.88"/>
   </cols>
   <sheetData>
@@ -735,430 +867,477 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="str">
+      <c r="A2" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A2) - 2)</f>
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>4</v>
+      <c r="B2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="str">
+      <c r="A3" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A3) - 2)</f>
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="B3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="str">
+      <c r="A4" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A4) - 2)</f>
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="B4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="str">
+      <c r="A5" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A5) - 2)</f>
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>10</v>
-      </c>
+      <c r="B5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="str">
+      <c r="A6" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A6) - 2)</f>
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="B6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="str">
+      <c r="A7" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A7) - 2)</f>
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="B7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="str">
+      <c r="A8" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A8) - 2)</f>
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>16</v>
+      <c r="B8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="str">
+      <c r="A9" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A9) - 2)</f>
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>18</v>
-      </c>
+      <c r="B9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="str">
+      <c r="A10" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A10) - 2)</f>
         <v>8</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>20</v>
-      </c>
+      <c r="B10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="str">
+      <c r="A11" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A11) - 2)</f>
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>22</v>
-      </c>
+      <c r="B11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="str">
+      <c r="A12" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A12) - 2)</f>
         <v>A</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>24</v>
-      </c>
+      <c r="B12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="str">
+      <c r="A13" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A13) - 2)</f>
         <v>B</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>26</v>
-      </c>
+      <c r="B13" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="str">
+      <c r="A14" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A14) - 2)</f>
         <v>C</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>28</v>
-      </c>
+      <c r="B14" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="str">
+      <c r="A15" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A15) - 2)</f>
         <v>D</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>30</v>
-      </c>
+      <c r="B15" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="str">
+      <c r="A16" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A16) - 2)</f>
         <v>E</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>32</v>
-      </c>
+      <c r="B16" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="str">
+      <c r="A17" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A17) - 2)</f>
         <v>F</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>34</v>
-      </c>
+      <c r="B17" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="str">
+      <c r="A18" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A18) - 2)</f>
         <v>10</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>36</v>
-      </c>
+      <c r="B18" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="str">
+      <c r="A19" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A19) - 2)</f>
         <v>11</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>38</v>
-      </c>
+      <c r="B19" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="str">
+      <c r="A20" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A20) - 2)</f>
         <v>12</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>40</v>
-      </c>
+      <c r="B20" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="str">
+      <c r="A21" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A21) - 2)</f>
         <v>13</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>42</v>
+      <c r="B21" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="str">
+      <c r="A22" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A22) - 2)</f>
         <v>14</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>44</v>
+      <c r="B22" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="str">
+      <c r="A23" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A23) - 2)</f>
         <v>15</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>46</v>
-      </c>
+      <c r="B23" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="str">
+      <c r="A24" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A24) - 2)</f>
         <v>16</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>48</v>
+      <c r="B24" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="str">
+      <c r="A25" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A25) - 2)</f>
         <v>17</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>50</v>
+      <c r="B25" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="str">
+      <c r="A26" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A26) - 2)</f>
         <v>18</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>52</v>
-      </c>
+      <c r="B26" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="str">
+      <c r="A27" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A27) - 2)</f>
         <v>19</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>54</v>
-      </c>
+      <c r="B27" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="str">
+      <c r="A28" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A28) - 2)</f>
         <v>1A</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>56</v>
-      </c>
+      <c r="B28" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="str">
+      <c r="A29" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A29) - 2)</f>
         <v>1B</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>58</v>
-      </c>
+      <c r="B29" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="str">
+      <c r="A30" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A30) - 2)</f>
         <v>1C</v>
       </c>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="str">
+      <c r="A31" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A31) - 2)</f>
         <v>1D</v>
       </c>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="str">
+      <c r="A32" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A32) - 2)</f>
         <v>1E</v>
       </c>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="str">
+      <c r="A33" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A33) - 2)</f>
         <v>1F</v>
       </c>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="str">
+      <c r="A34" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A34) - 2)</f>
         <v>20</v>
       </c>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="str">
+      <c r="A35" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A35) - 2)</f>
         <v>21</v>
       </c>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="str">
+      <c r="A36" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A36) - 2)</f>
         <v>22</v>
       </c>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
     </row>
     <row r="37" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3" t="str">
+      <c r="A37" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A37) - 2)</f>
         <v>23</v>
       </c>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="str">
+      <c r="A38" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A38) - 2)</f>
         <v>24</v>
       </c>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="str">
+      <c r="A39" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A39) - 2)</f>
         <v>25</v>
       </c>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
+      <c r="B39" s="5"/>
+      <c r="C39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="str">
+      <c r="A40" s="4" t="str">
         <f aca="false">DEC2HEX(ROW(A40) - 2)</f>
         <v>26</v>
       </c>
-      <c r="B40" s="4"/>
-      <c r="C40" s="4"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1191,239 +1370,239 @@
   <sheetData>
     <row r="1" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A2) - 2)</f>
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D2" s="4" t="n">
+      <c r="B2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>66</v>
+      <c r="E2" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="str">
+      <c r="A3" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A3) - 2)</f>
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D3" s="4" t="n">
+      <c r="B3" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>66</v>
+      <c r="E3" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="str">
+      <c r="A4" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A4) - 2)</f>
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="B4" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>66</v>
+      <c r="E4" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="str">
+      <c r="A5" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A5) - 2)</f>
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="4" t="n">
+      <c r="B5" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>66</v>
+      <c r="E5" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="str">
+      <c r="A6" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A6) - 2)</f>
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="B6" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>66</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="str">
+      <c r="A7" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A7) - 2)</f>
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D7" s="4" t="n">
+      <c r="B7" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>66</v>
+      <c r="E7" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="str">
+      <c r="A8" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A8) - 2)</f>
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="D8" s="4" t="n">
+      <c r="B8" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>66</v>
+      <c r="E8" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="str">
+      <c r="A9" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A9) - 2)</f>
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D9" s="4" t="n">
+      <c r="B9" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>81</v>
+      <c r="E9" s="5" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="str">
+      <c r="A10" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A10) - 2)</f>
         <v>8</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D10" s="4" t="n">
+      <c r="B10" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D10" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>81</v>
+      <c r="E10" s="5" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="str">
+      <c r="A11" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A11) - 2)</f>
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D11" s="4" t="n">
+      <c r="B11" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D11" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>81</v>
+      <c r="E11" s="5" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="str">
+      <c r="A12" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A12) - 2)</f>
         <v>A</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D12" s="4" t="n">
+      <c r="B12" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D12" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>81</v>
+      <c r="E12" s="5" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="str">
+      <c r="A13" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A13) - 2)</f>
         <v>B</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="D13" s="4" t="n">
+      <c r="B13" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D13" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>90</v>
+      <c r="E13" s="5" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="str">
+      <c r="A14" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A14) - 2)</f>
         <v>C</v>
       </c>
@@ -1433,7 +1612,7 @@
       <c r="E14" s="7"/>
     </row>
     <row r="15" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="str">
+      <c r="A15" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A15) - 2)</f>
         <v>D</v>
       </c>
@@ -1443,25 +1622,25 @@
       <c r="E15" s="7"/>
     </row>
     <row r="16" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="str">
+      <c r="A16" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A16) - 2)</f>
         <v>E</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D16" s="4" t="n">
+      <c r="B16" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>90</v>
+      <c r="E16" s="5" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="str">
+      <c r="A17" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A17) - 2)</f>
         <v>F</v>
       </c>
@@ -1471,7 +1650,7 @@
       <c r="E17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="str">
+      <c r="A18" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A18) - 2)</f>
         <v>10</v>
       </c>
@@ -1481,7 +1660,7 @@
       <c r="E18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="str">
+      <c r="A19" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A19) - 2)</f>
         <v>11</v>
       </c>
@@ -1491,228 +1670,244 @@
       <c r="E19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="str">
+      <c r="A20" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A20) - 2)</f>
         <v>12</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D20" s="4" t="n">
+      <c r="B20" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D20" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E20" s="4" t="s">
-        <v>95</v>
+      <c r="E20" s="5" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="str">
+      <c r="A21" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A21) - 2)</f>
         <v>13</v>
       </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
+      <c r="B21" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="str">
+      <c r="A22" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A22) - 2)</f>
         <v>14</v>
       </c>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="str">
+      <c r="A23" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A23) - 2)</f>
         <v>15</v>
       </c>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="E23" s="4"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="E23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="str">
+      <c r="A24" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A24) - 2)</f>
         <v>16</v>
       </c>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="str">
+      <c r="A25" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A25) - 2)</f>
         <v>17</v>
       </c>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="str">
+      <c r="A26" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A26) - 2)</f>
         <v>18</v>
       </c>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="str">
+      <c r="A27" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A27) - 2)</f>
         <v>19</v>
       </c>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="str">
+      <c r="A28" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A28) - 2)</f>
         <v>1A</v>
       </c>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="str">
+      <c r="A29" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A29) - 2)</f>
         <v>1B</v>
       </c>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="str">
+      <c r="A30" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A30) - 2)</f>
         <v>1C</v>
       </c>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="str">
+      <c r="A31" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A31) - 2)</f>
         <v>1D</v>
       </c>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="str">
+      <c r="A32" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A32) - 2)</f>
         <v>1E</v>
       </c>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="str">
+      <c r="A33" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A33) - 2)</f>
         <v>1F</v>
       </c>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="str">
+      <c r="A34" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A34) - 2)</f>
         <v>20</v>
       </c>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="str">
+      <c r="A35" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A35) - 2)</f>
         <v>21</v>
       </c>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="str">
+      <c r="A36" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A36) - 2)</f>
         <v>22</v>
       </c>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
     </row>
     <row r="37" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="str">
+      <c r="A37" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A37) - 2)</f>
         <v>23</v>
       </c>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="str">
+      <c r="A38" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A38) - 2)</f>
         <v>24</v>
       </c>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="str">
+      <c r="A39" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A39) - 2)</f>
         <v>25</v>
       </c>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="B39" s="5"/>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="str">
+      <c r="A40" s="5" t="str">
         <f aca="false">DEC2HEX(ROW(Operations!A40) - 2)</f>
         <v>26</v>
       </c>
-      <c r="B40" s="4"/>
-      <c r="C40" s="4"/>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E40" type="list">
+  <dataValidations count="3">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E21:E40" type="list">
+      <formula1>"Read,Write,None,Unknown,N/A"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E20" type="none">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E19" type="list">
       <formula1>"Read,Write,None,Unknown,N/A"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>